<commit_message>
Relabel projects 05-06 and template
</commit_message>
<xml_diff>
--- a/05-iso27001-readiness-soa/05-iso27001-readiness-and-soa.xlsx
+++ b/05-iso27001-readiness-soa/05-iso27001-readiness-and-soa.xlsx
@@ -40,7 +40,7 @@
     <t xml:space="preserve">CGI-ISO-001 — ISO/IEC 27001:2022 Readiness Assessment &amp; Statement of Applicability</t>
   </si>
   <si>
-    <t xml:space="preserve">FICTIONAL DATA - Cypher Group Inc. is not a real company. CGI-ISO-001 v1.0, 16 Sep 2026. Prepared by O.S; for approval by Jerry Olugboye.</t>
+    <t xml:space="preserve">SIMULATED CASE STUDY - Cypher Group Inc. is a simulated company. CGI-ISO-001 v1.0, 16 Sep 2026. Prepared by O.S; for approval by Jerry Olugboye.</t>
   </si>
   <si>
     <t xml:space="preserve">Item</t>
@@ -55,7 +55,7 @@
     <t xml:space="preserve">Readiness assessment and 93-control Statement of Applicability for Cypher Group Inc., tracing every control to CGI-RSK-001 v1.1, CGI-GAP-001 and CGI-TPR-001.</t>
   </si>
   <si>
-    <t xml:space="preserve">Fictional-data notice</t>
+    <t xml:space="preserve">Case-study notice</t>
   </si>
   <si>
     <t xml:space="preserve">All organisations, people, findings, scores, dates and costs are invented for a portfolio. Real product names are stand-ins; any assurance status attributed to them is invented. ISO wording is paraphrased.</t>
@@ -3940,7 +3940,7 @@
     <t xml:space="preserve">Target dates all after 16 Sep 2026</t>
   </si>
   <si>
-    <t xml:space="preserve">Fictional-data notice on every sheet</t>
+    <t xml:space="preserve">Case-study notice on every sheet</t>
   </si>
   <si>
     <t xml:space="preserve">Row 2 of every sheet</t>

</xml_diff>

<commit_message>
v1.4a fix: restore the CIS AWS Foundations Benchmark name
The rename pass turned three short references to the published CIS
benchmark into "CIS CloudCo". Benchmark titles keep their real name;
only supplier names are simulated. Projects 03, 05 and 06 md, csv, xlsx
and pdf corrected; workbooks recalculated with 0 formula errors.

Claude-Session: https://claude.ai/code/session_01FAKSHwJq6cPsfsijKdihQk
</commit_message>
<xml_diff>
--- a/05-iso27001-readiness-soa/05-iso27001-readiness-and-soa.xlsx
+++ b/05-iso27001-readiness-soa/05-iso27001-readiness-and-soa.xlsx
@@ -1585,7 +1585,7 @@
     <t xml:space="preserve">CG-03: there is no CloudCo configuration baseline and no drift detection (PR.IR = 0). This is the documented reason R-005 stays High.</t>
   </si>
   <si>
-    <t xml:space="preserve">Held: none. Required: CIS CloudCo Foundations baseline; posture-monitoring reports.</t>
+    <t xml:space="preserve">Held: none. Required: CIS AWS Foundations baseline; posture-monitoring reports.</t>
   </si>
   <si>
     <t xml:space="preserve">R-005; R-004</t>
@@ -3397,7 +3397,7 @@
     <t xml:space="preserve">The REC-10 agenda (KRIs, scorecard, TP status) is not a full clause 9.3 review. Extend it to the 9.3.2 a) to g) inputs and minute it as the management review.</t>
   </si>
   <si>
-    <t xml:space="preserve">CIS CloudCo baseline; posture monitoring</t>
+    <t xml:space="preserve">CIS AWS baseline; posture monitoring</t>
   </si>
   <si>
     <t xml:space="preserve">Q2 2027</t>

</xml_diff>